<commit_message>
Allow several new text col to appear in the tab for editting
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -698,7 +698,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -708,12 +708,12 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -763,7 +763,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR2" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -818,7 +822,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -828,12 +832,12 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -883,7 +887,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR3" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -934,7 +942,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -944,12 +952,12 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -999,7 +1007,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR4" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1046,7 +1058,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1056,12 +1068,12 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1111,7 +1123,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR5" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1162,7 +1178,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1172,12 +1188,12 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1227,7 +1243,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR6" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1282,7 +1302,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1292,12 +1312,12 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1347,7 +1367,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR7" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1402,7 +1426,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1412,12 +1436,12 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1467,7 +1491,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR8" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1522,7 +1550,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1532,12 +1560,12 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1587,7 +1615,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR9" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1642,7 +1674,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1652,12 +1684,12 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1707,7 +1739,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR10" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1758,7 +1794,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1768,12 +1804,12 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1823,7 +1859,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR11" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1870,7 +1910,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1880,12 +1920,12 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -1935,7 +1975,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR12" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1986,7 +2030,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1996,12 +2040,12 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2051,7 +2095,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR13" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2106,7 +2154,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2116,12 +2164,12 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2171,7 +2219,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR14" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2226,7 +2278,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2236,12 +2288,12 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2291,7 +2343,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR15" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2346,7 +2402,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2356,12 +2412,12 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2411,7 +2467,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR16" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2466,7 +2526,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2476,12 +2536,12 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2531,7 +2591,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR17" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2586,7 +2650,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2596,12 +2660,12 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2651,7 +2715,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR18" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2706,7 +2774,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2716,12 +2784,12 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -2771,7 +2839,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR19" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2826,7 +2898,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2836,12 +2908,12 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -2891,7 +2963,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ20" t="inlineStr"/>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR20" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2946,7 +3022,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -2956,12 +3032,12 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -3011,7 +3087,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR21" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3066,7 +3146,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -3076,12 +3156,12 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3131,7 +3211,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ22" t="inlineStr"/>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR22" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3186,7 +3270,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -3196,12 +3280,12 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -3251,7 +3335,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ23" t="inlineStr"/>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR23" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3306,7 +3394,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -3316,12 +3404,12 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3371,7 +3459,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ24" t="inlineStr"/>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR24" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3426,7 +3518,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -3436,12 +3528,12 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3491,7 +3583,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ25" t="inlineStr"/>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR25" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3546,7 +3642,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -3556,12 +3652,12 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -3611,7 +3707,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ26" t="inlineStr"/>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR26" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3666,7 +3766,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>IGAP + UKBB + UKBEC + ADNI + NABEC + ADGC + ADSP + CHARGE</t>
+          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -3676,12 +3776,12 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + 1000 Genomes + TOPMed + UK10K</t>
+          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>IGAP + 1000 Genomes EUR + European + ADGC + ADSP</t>
+          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
@@ -3731,7 +3831,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AQ27" t="inlineStr"/>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AR27" t="inlineStr">
         <is>
           <t>Table 1</t>

</xml_diff>

<commit_message>
Update code to fully run on new version of text col
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -685,7 +685,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -708,12 +708,12 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -809,7 +809,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -822,7 +822,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -832,12 +832,12 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -929,7 +929,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -952,12 +952,12 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1045,7 +1045,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1068,12 +1068,12 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1165,7 +1165,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1188,12 +1188,12 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1289,7 +1289,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1312,12 +1312,12 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1413,7 +1413,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1436,12 +1436,12 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1537,7 +1537,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1560,12 +1560,12 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1661,7 +1661,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1684,12 +1684,12 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1781,7 +1781,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1804,12 +1804,12 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1897,7 +1897,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1920,12 +1920,12 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2017,7 +2017,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -2040,12 +2040,12 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2141,7 +2141,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2164,12 +2164,12 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2265,7 +2265,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2288,12 +2288,12 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2389,7 +2389,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2412,12 +2412,12 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2513,7 +2513,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2536,12 +2536,12 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2637,7 +2637,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2660,12 +2660,12 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2761,7 +2761,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -2774,7 +2774,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2784,12 +2784,12 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -2885,7 +2885,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2908,12 +2908,12 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -3009,7 +3009,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -3032,12 +3032,12 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -3133,7 +3133,7 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -3156,12 +3156,12 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3257,7 +3257,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -3280,12 +3280,12 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -3381,7 +3381,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -3404,12 +3404,12 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3505,7 +3505,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -3528,12 +3528,12 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3629,7 +3629,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -3652,12 +3652,12 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -3753,7 +3753,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Discovery + Meta-analysis + IGAP</t>
+          <t>IGAP + Discovery + Meta-analysis</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>IGAP + CHARGE + ADNI + UKBB + NABEC + ADGC + ADSP + UKBEC</t>
+          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -3776,12 +3776,12 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1000 Genomes + UK10K + TOPMed + Haplotype Reference Consortium</t>
+          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + IGAP + ADGC + ADSP + European</t>
+          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>

</xml_diff>

<commit_message>
reduce amount text generated + allow pipeline to run on cpu + combine with Sherry's current pipeline
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT27"/>
+  <dimension ref="A1:AT19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -663,7 +663,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CR1</t>
+          <t>rs4844600</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -685,7 +685,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -708,20 +708,16 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -732,14 +728,12 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>rs6656401</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="n">
-        <v>8.489999999999999e-07</v>
-      </c>
+      <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
@@ -749,12 +743,10 @@
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL2" t="n">
-        <v>1.17</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr"/>
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
@@ -787,7 +779,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CR1</t>
+          <t>rs6656401</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -809,7 +801,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -822,7 +814,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -832,20 +824,16 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -856,14 +844,12 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>rs4844600</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="n">
-        <v>4.219999999999999e-07</v>
-      </c>
+      <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
@@ -873,12 +859,10 @@
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL3" t="n">
-        <v>1.17</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr"/>
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
@@ -909,7 +893,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>rs2296160</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>30448613_table1_R00003</t>
@@ -929,7 +917,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -942,7 +930,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -952,20 +940,16 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -976,14 +960,12 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>rs2296160</t>
+          <t>8.56×10 −3</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="n">
-        <v>4.24e-08</v>
-      </c>
+      <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
@@ -993,12 +975,10 @@
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL4" t="n">
-        <v>1.18</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr"/>
@@ -1022,10 +1002,18 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>CR1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>rs9270303</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>30448613_table1_R00004</t>
@@ -1045,7 +1033,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1058,7 +1046,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1068,20 +1056,16 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1092,14 +1076,12 @@
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>rs2296160</t>
+          <t>2.50×10 −4</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="n">
-        <v>0.00856</v>
-      </c>
+      <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
@@ -1109,12 +1091,10 @@
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL5" t="n">
-        <v>1.11</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
@@ -1138,12 +1118,16 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>HLA-DRB5</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HLA-DRB5</t>
+          <t>rs9271192</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1165,7 +1149,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1178,7 +1162,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1188,20 +1172,16 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1212,14 +1192,12 @@
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>rs9271192</t>
+          <t>2.50×10 −4</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="n">
-        <v>0.000266</v>
-      </c>
+      <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
@@ -1229,12 +1207,10 @@
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL6" t="n">
-        <v>1.11</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
@@ -1267,7 +1243,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HLA-DRB5</t>
+          <t>rs1476679</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1289,7 +1265,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1302,7 +1278,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1312,20 +1288,16 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1336,14 +1308,12 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>rs9270303</t>
+          <t>1.09×10 −3</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="n">
-        <v>0.00025</v>
-      </c>
+      <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
@@ -1353,12 +1323,10 @@
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL7" t="n">
-        <v>1.15</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
@@ -1384,14 +1352,14 @@
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>HLA-DRB5</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>rs2405442</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1413,7 +1381,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1426,7 +1394,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1436,20 +1404,16 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1460,14 +1424,12 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>rs1476679</t>
+          <t>1.09×10 −3</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="n">
-        <v>0.00141</v>
-      </c>
+      <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
@@ -1477,12 +1439,10 @@
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL8" t="n">
-        <v>0.92</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
@@ -1515,7 +1475,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>rs1859788</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1537,7 +1497,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1550,7 +1510,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1560,20 +1520,16 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1584,14 +1540,12 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>rs2405442</t>
+          <t>1.12×10 −3</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="n">
-        <v>0.00212</v>
-      </c>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
@@ -1601,12 +1555,10 @@
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL9" t="n">
-        <v>0.92</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
@@ -1639,7 +1591,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>rs7982</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1661,7 +1613,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1674,7 +1626,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1684,20 +1636,16 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1708,14 +1656,12 @@
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>rs2405442</t>
+          <t>1.62×10 −3</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="n">
-        <v>0.00109</v>
-      </c>
+      <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
@@ -1725,12 +1671,10 @@
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL10" t="n">
-        <v>0.89</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr"/>
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
@@ -1756,12 +1700,16 @@
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>CLU</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>rs9331896</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>30448613_table1_R00010</t>
@@ -1781,7 +1729,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1794,7 +1742,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1804,20 +1752,16 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1828,14 +1772,12 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>rs1859788</t>
+          <t>1.62×10 −3</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="n">
-        <v>0.00562</v>
-      </c>
+      <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
@@ -1845,12 +1787,10 @@
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL11" t="n">
-        <v>0.93</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
@@ -1874,10 +1814,18 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>CLU</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>rs10838725</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>30448613_table1_R00011</t>
@@ -1897,7 +1845,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1910,7 +1858,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1920,20 +1868,16 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -1944,14 +1888,12 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>rs1859788</t>
+          <t>0.040</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="n">
-        <v>0.00112</v>
-      </c>
+      <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
@@ -1961,12 +1903,10 @@
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL12" t="n">
-        <v>0.89</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr"/>
       <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
@@ -1990,12 +1930,16 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>CELF1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>rs2293576</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2017,7 +1961,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2030,7 +1974,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -2040,20 +1984,16 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -2064,14 +2004,12 @@
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>rs9331896</t>
+          <t>0.040</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="n">
-        <v>0.00102</v>
-      </c>
+      <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
@@ -2081,12 +2019,10 @@
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL13" t="n">
-        <v>0.92</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr"/>
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
@@ -2112,14 +2048,14 @@
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>CELF1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>rs12453</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2141,7 +2077,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2154,7 +2090,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2164,20 +2100,16 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -2188,14 +2120,12 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>rs7982</t>
+          <t>3.60×10 −4</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="n">
-        <v>0.000364</v>
-      </c>
+      <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
@@ -2205,12 +2135,10 @@
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL14" t="n">
-        <v>0.91</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr"/>
       <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
@@ -2236,14 +2164,14 @@
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>MS4A6A</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>rs983392</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2265,7 +2193,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2278,7 +2206,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2288,20 +2216,16 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -2312,14 +2236,12 @@
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>rs7982</t>
+          <t>3.60×10 −4</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="n">
-        <v>0.00162</v>
-      </c>
+      <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
@@ -2329,12 +2251,10 @@
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL15" t="n">
-        <v>0.9</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr"/>
       <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
@@ -2360,14 +2280,14 @@
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>MS4A6A</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>rs3752246</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2389,7 +2309,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2402,7 +2322,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2412,20 +2332,16 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -2436,14 +2352,12 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>rs10838725</t>
+          <t>9.89×10 −5</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="n">
-        <v>0.054</v>
-      </c>
+      <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
@@ -2453,12 +2367,10 @@
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL16" t="n">
-        <v>1.05</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr"/>
       <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr"/>
@@ -2484,14 +2396,14 @@
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>ABCA7</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>rs4147929</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2513,7 +2425,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2526,7 +2438,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2536,20 +2448,16 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -2560,14 +2468,12 @@
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>rs2293576</t>
+          <t>9.89×10 −5</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="n">
-        <v>0.24</v>
-      </c>
+      <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr"/>
@@ -2577,12 +2483,10 @@
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL17" t="n">
-        <v>1.03</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr"/>
       <c r="AM17" t="inlineStr"/>
       <c r="AN17" t="inlineStr"/>
       <c r="AO17" t="inlineStr"/>
@@ -2608,14 +2512,14 @@
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>ABCA7</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>rs12459419</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2637,7 +2541,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -2650,7 +2554,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2660,20 +2564,16 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
+      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -2684,14 +2584,12 @@
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>rs2293576</t>
+          <t>0.090</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="n">
-        <v>0.04</v>
-      </c>
+      <c r="AC18" t="inlineStr"/>
       <c r="AD18" t="inlineStr"/>
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
@@ -2701,12 +2599,10 @@
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL18" t="n">
-        <v>1.07</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr"/>
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr"/>
@@ -2732,14 +2628,14 @@
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>CD33</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MS4A6A</t>
+          <t>rs3865444</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2761,7 +2657,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
+          <t>Discovery + IGAP + Meta-analysis</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -2774,7 +2670,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
+          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2784,20 +2680,16 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
+          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
+          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
           <t>Alzheimer's disease + AD</t>
@@ -2808,14 +2700,12 @@
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>rs983392</t>
+          <t>0.090</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="n">
-        <v>7.22e-09</v>
-      </c>
+      <c r="AC19" t="inlineStr"/>
       <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
@@ -2825,12 +2715,10 @@
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL19" t="n">
-        <v>0.86</v>
-      </c>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr"/>
       <c r="AM19" t="inlineStr"/>
       <c r="AN19" t="inlineStr"/>
       <c r="AO19" t="inlineStr"/>
@@ -2855,998 +2743,6 @@
         </is>
       </c>
       <c r="AT19" t="inlineStr">
-        <is>
-          <t>MS4A6A</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>MS4A6A</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00019</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>rs12453</t>
-        </is>
-      </c>
-      <c r="AA20" t="inlineStr"/>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="n">
-        <v>1.34e-09</v>
-      </c>
-      <c r="AD20" t="inlineStr"/>
-      <c r="AE20" t="inlineStr"/>
-      <c r="AF20" t="inlineStr"/>
-      <c r="AG20" t="inlineStr"/>
-      <c r="AH20" t="inlineStr"/>
-      <c r="AI20" t="inlineStr"/>
-      <c r="AJ20" t="inlineStr"/>
-      <c r="AK20" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL20" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="AM20" t="inlineStr"/>
-      <c r="AN20" t="inlineStr"/>
-      <c r="AO20" t="inlineStr"/>
-      <c r="AP20" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ20" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR20" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS20" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT20" t="inlineStr">
-        <is>
-          <t>MS4A6A</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>MS4A6A</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00020</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr">
-        <is>
-          <t>rs12453</t>
-        </is>
-      </c>
-      <c r="AA21" t="inlineStr"/>
-      <c r="AB21" t="inlineStr"/>
-      <c r="AC21" t="n">
-        <v>0.00036</v>
-      </c>
-      <c r="AD21" t="inlineStr"/>
-      <c r="AE21" t="inlineStr"/>
-      <c r="AF21" t="inlineStr"/>
-      <c r="AG21" t="inlineStr"/>
-      <c r="AH21" t="inlineStr"/>
-      <c r="AI21" t="inlineStr"/>
-      <c r="AJ21" t="inlineStr"/>
-      <c r="AK21" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL21" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="AM21" t="inlineStr"/>
-      <c r="AN21" t="inlineStr"/>
-      <c r="AO21" t="inlineStr"/>
-      <c r="AP21" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ21" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR21" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS21" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT21" t="inlineStr">
-        <is>
-          <t>MS4A6A</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ABCA7</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00021</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr">
-        <is>
-          <t>rs4147929</t>
-        </is>
-      </c>
-      <c r="AA22" t="inlineStr"/>
-      <c r="AB22" t="inlineStr"/>
-      <c r="AC22" t="n">
-        <v>0.00139</v>
-      </c>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
-      <c r="AF22" t="inlineStr"/>
-      <c r="AG22" t="inlineStr"/>
-      <c r="AH22" t="inlineStr"/>
-      <c r="AI22" t="inlineStr"/>
-      <c r="AJ22" t="inlineStr"/>
-      <c r="AK22" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL22" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="AM22" t="inlineStr"/>
-      <c r="AN22" t="inlineStr"/>
-      <c r="AO22" t="inlineStr"/>
-      <c r="AP22" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ22" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR22" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS22" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT22" t="inlineStr">
-        <is>
-          <t>ABCA7</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ABCA7</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00022</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>rs3752246</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="n">
-        <v>0.0027</v>
-      </c>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
-      <c r="AF23" t="inlineStr"/>
-      <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr"/>
-      <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
-      <c r="AK23" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL23" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="AM23" t="inlineStr"/>
-      <c r="AN23" t="inlineStr"/>
-      <c r="AO23" t="inlineStr"/>
-      <c r="AP23" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ23" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR23" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS23" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT23" t="inlineStr">
-        <is>
-          <t>ABCA7</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ABCA7</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00023</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr">
-        <is>
-          <t>rs3752246</t>
-        </is>
-      </c>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="n">
-        <v>9.890000000000002e-05</v>
-      </c>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr"/>
-      <c r="AF24" t="inlineStr"/>
-      <c r="AG24" t="inlineStr"/>
-      <c r="AH24" t="inlineStr"/>
-      <c r="AI24" t="inlineStr"/>
-      <c r="AJ24" t="inlineStr"/>
-      <c r="AK24" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL24" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="AM24" t="inlineStr"/>
-      <c r="AN24" t="inlineStr"/>
-      <c r="AO24" t="inlineStr"/>
-      <c r="AP24" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ24" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR24" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS24" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT24" t="inlineStr">
-        <is>
-          <t>ABCA7</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>CD33</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00024</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr">
-        <is>
-          <t>rs3865444</t>
-        </is>
-      </c>
-      <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="n">
-        <v>0.000449</v>
-      </c>
-      <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="inlineStr"/>
-      <c r="AF25" t="inlineStr"/>
-      <c r="AG25" t="inlineStr"/>
-      <c r="AH25" t="inlineStr"/>
-      <c r="AI25" t="inlineStr"/>
-      <c r="AJ25" t="inlineStr"/>
-      <c r="AK25" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL25" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="AM25" t="inlineStr"/>
-      <c r="AN25" t="inlineStr"/>
-      <c r="AO25" t="inlineStr"/>
-      <c r="AP25" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ25" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR25" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS25" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT25" t="inlineStr">
-        <is>
-          <t>CD33</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>CD33</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00025</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>rs12459419</t>
-        </is>
-      </c>
-      <c r="AA26" t="inlineStr"/>
-      <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="n">
-        <v>0.000402</v>
-      </c>
-      <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
-      <c r="AF26" t="inlineStr"/>
-      <c r="AG26" t="inlineStr"/>
-      <c r="AH26" t="inlineStr"/>
-      <c r="AI26" t="inlineStr"/>
-      <c r="AJ26" t="inlineStr"/>
-      <c r="AK26" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL26" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="AM26" t="inlineStr"/>
-      <c r="AN26" t="inlineStr"/>
-      <c r="AO26" t="inlineStr"/>
-      <c r="AP26" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ26" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR26" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS26" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT26" t="inlineStr">
-        <is>
-          <t>CD33</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>CD33</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>30448613_table1_R00026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>30448613_table1</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>T00001</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>IGAP + Discovery + Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>SNP-based</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>IGAP + NABEC + ADSP + ADNI + UKBEC + CHARGE + UKBB + ADGC</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Haplotype Reference Consortium + UK10K + TOPMed + 1000 Genomes</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>IGAP + ADSP + European + 1000 Genomes EUR + ADGC</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>Alzheimer's disease + AD</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>rs12459419</t>
-        </is>
-      </c>
-      <c r="AA27" t="inlineStr"/>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="AD27" t="inlineStr"/>
-      <c r="AE27" t="inlineStr"/>
-      <c r="AF27" t="inlineStr"/>
-      <c r="AG27" t="inlineStr"/>
-      <c r="AH27" t="inlineStr"/>
-      <c r="AI27" t="inlineStr"/>
-      <c r="AJ27" t="inlineStr"/>
-      <c r="AK27" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="AL27" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="AM27" t="inlineStr"/>
-      <c r="AN27" t="inlineStr"/>
-      <c r="AO27" t="inlineStr"/>
-      <c r="AP27" t="inlineStr">
-        <is>
-          <t>30448613</t>
-        </is>
-      </c>
-      <c r="AQ27" t="inlineStr">
-        <is>
-          <t>PMC6331247</t>
-        </is>
-      </c>
-      <c r="AR27" t="inlineStr">
-        <is>
-          <t>Table 1</t>
-        </is>
-      </c>
-      <c r="AS27" t="inlineStr">
-        <is>
-          <t>30448613_table1.xlsx</t>
-        </is>
-      </c>
-      <c r="AT27" t="inlineStr">
         <is>
           <t>CD33</t>
         </is>

</xml_diff>

<commit_message>
Update to a more lightweight llm  + require less max text generated
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT19"/>
+  <dimension ref="A1:AT27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -663,7 +663,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>rs4844600</t>
+          <t>CR1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -685,7 +685,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -708,19 +708,23 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -728,12 +732,14 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rs6656401</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+      <c r="AC2" t="n">
+        <v>8.489999999999999e-07</v>
+      </c>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
@@ -743,10 +749,12 @@
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL2" t="n">
+        <v>1.17</v>
+      </c>
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
@@ -779,7 +787,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rs6656401</t>
+          <t>CR1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -801,7 +809,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -814,7 +822,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -824,19 +832,23 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -844,12 +856,14 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>rs4844600</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
+      <c r="AC3" t="n">
+        <v>4.219999999999999e-07</v>
+      </c>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
@@ -859,10 +873,12 @@
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL3" t="n">
+        <v>1.17</v>
+      </c>
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr"/>
@@ -893,11 +909,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>rs2296160</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>30448613_table1_R00003</t>
@@ -917,7 +929,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -930,7 +942,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -940,19 +952,23 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -960,12 +976,14 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>8.56×10 −3</t>
+          <t>rs2296160</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AC4" t="n">
+        <v>4.24e-08</v>
+      </c>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
@@ -975,10 +993,12 @@
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL4" t="n">
+        <v>1.18</v>
+      </c>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr"/>
@@ -1002,18 +1022,10 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr">
-        <is>
-          <t>CR1</t>
-        </is>
-      </c>
+      <c r="AT4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>rs9270303</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>30448613_table1_R00004</t>
@@ -1033,7 +1045,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1046,7 +1058,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1056,19 +1068,23 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -1076,12 +1092,14 @@
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>2.50×10 −4</t>
+          <t>rs2296160</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
+      <c r="AC5" t="n">
+        <v>0.00856</v>
+      </c>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
@@ -1091,10 +1109,12 @@
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL5" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL5" t="n">
+        <v>1.11</v>
+      </c>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
@@ -1118,16 +1138,12 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>HLA-DRB5</t>
-        </is>
-      </c>
+      <c r="AT5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rs9271192</t>
+          <t>HLA-DRB5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1149,7 +1165,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1162,7 +1178,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1172,19 +1188,23 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -1192,12 +1212,14 @@
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>2.50×10 −4</t>
+          <t>rs9271192</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
+      <c r="AC6" t="n">
+        <v>0.000266</v>
+      </c>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
@@ -1207,10 +1229,12 @@
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL6" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL6" t="n">
+        <v>1.11</v>
+      </c>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
@@ -1243,7 +1267,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rs1476679</t>
+          <t>HLA-DRB5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1265,7 +1289,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1278,7 +1302,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1288,19 +1312,23 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1308,12 +1336,14 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>1.09×10 −3</t>
+          <t>rs9270303</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
+      <c r="AC7" t="n">
+        <v>0.00025</v>
+      </c>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
@@ -1323,10 +1353,12 @@
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL7" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL7" t="n">
+        <v>1.15</v>
+      </c>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
@@ -1352,14 +1384,14 @@
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>HLA-DRB5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rs2405442</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1381,7 +1413,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1394,7 +1426,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1404,19 +1436,23 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1424,12 +1460,14 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>1.09×10 −3</t>
+          <t>rs1476679</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
+      <c r="AC8" t="n">
+        <v>0.00141</v>
+      </c>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
@@ -1439,10 +1477,12 @@
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL8" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL8" t="n">
+        <v>0.92</v>
+      </c>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
@@ -1475,7 +1515,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rs1859788</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1497,7 +1537,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1510,7 +1550,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1520,19 +1560,23 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1540,12 +1584,14 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>1.12×10 −3</t>
+          <t>rs2405442</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+      <c r="AC9" t="n">
+        <v>0.00212</v>
+      </c>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
@@ -1555,10 +1601,12 @@
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL9" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.92</v>
+      </c>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
@@ -1591,7 +1639,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rs7982</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1613,7 +1661,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1626,7 +1674,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1636,19 +1684,23 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1656,12 +1708,14 @@
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>1.62×10 −3</t>
+          <t>rs2405442</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+      <c r="AC10" t="n">
+        <v>0.00109</v>
+      </c>
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
@@ -1671,10 +1725,12 @@
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL10" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL10" t="n">
+        <v>0.89</v>
+      </c>
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
@@ -1700,16 +1756,12 @@
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>rs9331896</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>30448613_table1_R00010</t>
@@ -1729,7 +1781,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1742,7 +1794,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1752,19 +1804,23 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1772,12 +1828,14 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>1.62×10 −3</t>
+          <t>rs1859788</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
+      <c r="AC11" t="n">
+        <v>0.00562</v>
+      </c>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
@@ -1787,10 +1845,12 @@
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL11" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.93</v>
+      </c>
       <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
@@ -1814,18 +1874,10 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT11" t="inlineStr">
-        <is>
-          <t>CLU</t>
-        </is>
-      </c>
+      <c r="AT11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>rs10838725</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>30448613_table1_R00011</t>
@@ -1845,7 +1897,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1858,7 +1910,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1868,19 +1920,23 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1888,12 +1944,14 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>0.040</t>
+          <t>rs1859788</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
+      <c r="AC12" t="n">
+        <v>0.00112</v>
+      </c>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
@@ -1903,10 +1961,12 @@
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL12" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL12" t="n">
+        <v>0.89</v>
+      </c>
       <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
@@ -1930,16 +1990,12 @@
           <t>30448613_table1.xlsx</t>
         </is>
       </c>
-      <c r="AT12" t="inlineStr">
-        <is>
-          <t>CELF1</t>
-        </is>
-      </c>
+      <c r="AT12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rs2293576</t>
+          <t>CLU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1961,7 +2017,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1974,7 +2030,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1984,19 +2040,23 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -2004,12 +2064,14 @@
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>0.040</t>
+          <t>rs9331896</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
+      <c r="AC13" t="n">
+        <v>0.00102</v>
+      </c>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
@@ -2019,10 +2081,12 @@
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL13" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL13" t="n">
+        <v>0.92</v>
+      </c>
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
@@ -2048,14 +2112,14 @@
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>CLU</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rs12453</t>
+          <t>CLU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2077,7 +2141,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2090,7 +2154,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2100,19 +2164,23 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -2120,12 +2188,14 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>3.60×10 −4</t>
+          <t>rs7982</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
+      <c r="AC14" t="n">
+        <v>0.000364</v>
+      </c>
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
@@ -2135,10 +2205,12 @@
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL14" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL14" t="n">
+        <v>0.91</v>
+      </c>
       <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
@@ -2164,14 +2236,14 @@
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>MS4A6A</t>
+          <t>CLU</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rs983392</t>
+          <t>CLU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2193,7 +2265,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2206,7 +2278,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2216,19 +2288,23 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -2236,12 +2312,14 @@
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>3.60×10 −4</t>
+          <t>rs7982</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
+      <c r="AC15" t="n">
+        <v>0.00162</v>
+      </c>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
@@ -2251,10 +2329,12 @@
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL15" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL15" t="n">
+        <v>0.9</v>
+      </c>
       <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
@@ -2280,14 +2360,14 @@
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>MS4A6A</t>
+          <t>CLU</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rs3752246</t>
+          <t>CELF1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2309,7 +2389,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2322,7 +2402,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2332,19 +2412,23 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -2352,12 +2436,14 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>9.89×10 −5</t>
+          <t>rs10838725</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
+      <c r="AC16" t="n">
+        <v>0.054</v>
+      </c>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
@@ -2367,10 +2453,12 @@
       <c r="AJ16" t="inlineStr"/>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL16" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL16" t="n">
+        <v>1.05</v>
+      </c>
       <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr"/>
@@ -2396,14 +2484,14 @@
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>ABCA7</t>
+          <t>CELF1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>rs4147929</t>
+          <t>CELF1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2425,7 +2513,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2438,7 +2526,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2448,19 +2536,23 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -2468,12 +2560,14 @@
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>9.89×10 −5</t>
+          <t>rs2293576</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
+      <c r="AC17" t="n">
+        <v>0.24</v>
+      </c>
       <c r="AD17" t="inlineStr"/>
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr"/>
@@ -2483,10 +2577,12 @@
       <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL17" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL17" t="n">
+        <v>1.03</v>
+      </c>
       <c r="AM17" t="inlineStr"/>
       <c r="AN17" t="inlineStr"/>
       <c r="AO17" t="inlineStr"/>
@@ -2512,14 +2608,14 @@
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>ABCA7</t>
+          <t>CELF1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>rs12459419</t>
+          <t>CELF1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2541,7 +2637,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -2554,7 +2650,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2564,19 +2660,23 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -2584,12 +2684,14 @@
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>0.090</t>
+          <t>rs2293576</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
+      <c r="AC18" t="n">
+        <v>0.04</v>
+      </c>
       <c r="AD18" t="inlineStr"/>
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
@@ -2599,10 +2701,12 @@
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL18" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL18" t="n">
+        <v>1.07</v>
+      </c>
       <c r="AM18" t="inlineStr"/>
       <c r="AN18" t="inlineStr"/>
       <c r="AO18" t="inlineStr"/>
@@ -2628,14 +2732,14 @@
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>CD33</t>
+          <t>CELF1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>rs3865444</t>
+          <t>MS4A6A</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2657,7 +2761,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Discovery + IGAP + Meta-analysis</t>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -2670,7 +2774,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>CHARGE + UKBEC + ADGC + NABEC + IGAP + ADSP + UKBB + ADNI</t>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2680,19 +2784,23 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>TOPMed + 1000 Genomes + UK10K + HRC;1000G + Haplotype Reference Consortium</t>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1000 Genomes EUR + ADGC + European ancestry + European + IGAP + ADSP</t>
+          <t>adgc + adsp + EUR + European ancestry</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Alzheimer's disease + AD</t>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -2700,12 +2808,14 @@
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>0.090</t>
+          <t>rs983392</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
+      <c r="AC19" t="n">
+        <v>7.22e-09</v>
+      </c>
       <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
@@ -2715,10 +2825,12 @@
       <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AL19" t="inlineStr"/>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL19" t="n">
+        <v>0.86</v>
+      </c>
       <c r="AM19" t="inlineStr"/>
       <c r="AN19" t="inlineStr"/>
       <c r="AO19" t="inlineStr"/>
@@ -2743,6 +2855,998 @@
         </is>
       </c>
       <c r="AT19" t="inlineStr">
+        <is>
+          <t>MS4A6A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MS4A6A</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00019</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>rs12453</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="n">
+        <v>1.34e-09</v>
+      </c>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL20" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AM20" t="inlineStr"/>
+      <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>MS4A6A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MS4A6A</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00020</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>rs12453</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="n">
+        <v>0.00036</v>
+      </c>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL21" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="AM21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>MS4A6A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ABCA7</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00021</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>rs4147929</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="n">
+        <v>0.00139</v>
+      </c>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="AM22" t="inlineStr"/>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>ABCA7</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ABCA7</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00022</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>rs3752246</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL23" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="AM23" t="inlineStr"/>
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>ABCA7</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ABCA7</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00023</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>rs3752246</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="n">
+        <v>9.890000000000002e-05</v>
+      </c>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL24" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>ABCA7</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CD33</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00024</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>rs3865444</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="n">
+        <v>0.000449</v>
+      </c>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL25" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AM25" t="inlineStr"/>
+      <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr"/>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>CD33</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CD33</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00025</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>ADGC</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>rs12459419</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="n">
+        <v>0.000402</v>
+      </c>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL26" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AM26" t="inlineStr"/>
+      <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="inlineStr"/>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>CD33</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CD33</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>30448613_table1_R00026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>30448613_table1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>T00001</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>SNP-based</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>adgc + adsp + EUR + European ancestry</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>ADSP</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>abca7 + ms4a6a + alzheimers disease</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>rs12459419</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr"/>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="AL27" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AM27" t="inlineStr"/>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>30448613</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>30448613_table1.xlsx</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
         <is>
           <t>CD33</t>
         </is>

</xml_diff>

<commit_message>
Adding cache for information dict of different paper based on pmid (=> 1 llm call per paper of multiple tables)
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -685,7 +685,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -708,12 +708,12 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -809,7 +809,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -822,7 +822,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -832,12 +832,12 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -929,7 +929,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -952,12 +952,12 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1045,7 +1045,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1068,12 +1068,12 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1165,7 +1165,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1188,12 +1188,12 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1289,7 +1289,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1312,12 +1312,12 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1413,7 +1413,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1436,12 +1436,12 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1537,7 +1537,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1560,12 +1560,12 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1661,7 +1661,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1684,12 +1684,12 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1781,7 +1781,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1804,12 +1804,12 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1897,7 +1897,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1920,12 +1920,12 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2017,7 +2017,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -2040,12 +2040,12 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2141,7 +2141,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2164,12 +2164,12 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2265,7 +2265,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2288,12 +2288,12 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2389,7 +2389,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2412,12 +2412,12 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2513,7 +2513,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2536,12 +2536,12 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2637,7 +2637,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2660,12 +2660,12 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2761,7 +2761,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -2774,7 +2774,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2784,12 +2784,12 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -2885,7 +2885,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2908,12 +2908,12 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -3009,7 +3009,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -3032,12 +3032,12 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -3133,7 +3133,7 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -3146,7 +3146,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -3156,12 +3156,12 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3257,7 +3257,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -3280,12 +3280,12 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -3381,7 +3381,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -3404,12 +3404,12 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3505,7 +3505,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -3528,12 +3528,12 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3629,7 +3629,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -3652,12 +3652,12 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -3753,7 +3753,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>replication + meta-analysis + Meta-analysis + discovery</t>
+          <t>replication + meta-analysis + discovery</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>IGAP + UKBEC + ADGC + CHARGE + ADNI + NABEC + ADSP + UKBB</t>
+          <t>ADGC + ADNI + NABEC + CHARGE + IGAP + UKBB + UKBEC + ADSP</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -3776,12 +3776,12 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>IGAP + UK10K + 1000G + HRC;1000G + HRC + TOPMed</t>
+          <t>topmed + igap + hrc + hrc;1000g + 1000g + uk10k</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>adgc + adsp + EUR + European ancestry</t>
+          <t>adsp + adgc + european ancestry + eur</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>

</xml_diff>

<commit_message>
add checking for weird terms in text columns
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,237 +429,237 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>RecordID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>PaperIDX</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>TableIDX</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Stage_original</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Analyses type</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Model type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Meta/Joint</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>SNP-based, Gene-based</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Cohort</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Cohort_simplified (no counts)</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Sample size</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Cases</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Controls</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Sample information</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Imputation_simple2</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Imputation</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Population_map</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Analysis group</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Phenotype</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Phenotype-derived</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>For plotting Beta and OR - derived</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Reported gene (gene based test)</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>TopSNP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Interactions</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Chr</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>P-value note</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>BP(Position)</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>RA 1(Reported Allele 1)</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>RA 2(Reported Allele 2)</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Note on alleles and AF</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>ReportedAF(MAF)</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>AFincases</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>AFincontrols</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Effect Size Type (OR or Beta)</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>EffectSize(altvsref)</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>95%ConfidenceInterval</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Confirmed affected genes, causal variants, evidence</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Genome build (hg18/hg37/hg38)</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Pubmed PMID</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>PMCID</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Table Ref in paper</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Table links</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>LocusName</t>
         </is>
@@ -675,31 +687,15 @@
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -707,30 +703,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -739,7 +727,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
@@ -777,7 +769,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS2" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -816,31 +812,15 @@
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -848,30 +828,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -880,7 +852,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
@@ -918,7 +894,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS3" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -953,31 +933,15 @@
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -985,30 +949,22 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1017,7 +973,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
@@ -1055,7 +1015,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS4" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1086,31 +1050,15 @@
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -1118,30 +1066,22 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1150,7 +1090,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
@@ -1188,7 +1132,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS5" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1223,31 +1171,15 @@
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -1255,30 +1187,22 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1287,7 +1211,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
@@ -1325,7 +1253,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS6" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1364,31 +1296,15 @@
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -1396,30 +1312,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1428,7 +1336,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
@@ -1466,7 +1378,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS7" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1505,31 +1421,15 @@
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -1537,30 +1437,22 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1569,7 +1461,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
@@ -1607,7 +1503,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS8" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1646,31 +1546,15 @@
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -1678,30 +1562,22 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1710,7 +1586,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
@@ -1748,7 +1628,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS9" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1787,31 +1671,15 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -1819,30 +1687,22 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1851,7 +1711,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
@@ -1889,7 +1753,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS10" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -1924,31 +1792,15 @@
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -1956,30 +1808,22 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1988,7 +1832,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
@@ -2026,7 +1874,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS11" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2057,31 +1909,15 @@
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -2089,30 +1925,22 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2121,7 +1949,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
@@ -2159,7 +1991,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS12" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2194,31 +2030,15 @@
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -2226,30 +2046,22 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2258,7 +2070,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
@@ -2296,7 +2112,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS13" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2335,31 +2155,15 @@
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -2367,30 +2171,22 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2399,7 +2195,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
@@ -2437,7 +2237,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS14" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2476,31 +2280,15 @@
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -2508,30 +2296,22 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2540,7 +2320,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
@@ -2578,7 +2362,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS15" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2617,31 +2405,15 @@
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -2649,30 +2421,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2681,7 +2445,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
@@ -2719,7 +2487,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS16" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2758,31 +2530,15 @@
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -2790,30 +2546,22 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2822,7 +2570,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
@@ -2860,7 +2612,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS17" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -2899,31 +2655,15 @@
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -2931,30 +2671,22 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2963,7 +2695,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
@@ -3001,7 +2737,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS18" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3040,31 +2780,15 @@
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -3072,30 +2796,22 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -3104,7 +2820,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
@@ -3142,7 +2862,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS19" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3181,31 +2905,15 @@
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -3213,30 +2921,22 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -3245,7 +2945,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
@@ -3283,7 +2987,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS20" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3322,31 +3030,15 @@
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -3354,30 +3046,22 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -3386,7 +3070,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr"/>
@@ -3424,7 +3112,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS21" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3463,31 +3155,15 @@
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -3495,30 +3171,22 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3527,7 +3195,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
@@ -3565,7 +3237,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR22" t="inlineStr"/>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS22" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3604,31 +3280,15 @@
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -3636,30 +3296,22 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -3668,7 +3320,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr"/>
@@ -3706,7 +3362,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS23" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3745,31 +3405,15 @@
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -3777,30 +3421,22 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3809,7 +3445,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr"/>
@@ -3847,7 +3487,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS24" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -3886,31 +3530,15 @@
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -3918,30 +3546,22 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>ADGC;IGAP</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3950,7 +3570,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
@@ -3988,7 +3612,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR25" t="inlineStr"/>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS25" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -4027,31 +3655,15 @@
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -4059,30 +3671,22 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>ADGC</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -4091,7 +3695,11 @@
           <t>ADGC</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr"/>
@@ -4129,7 +3737,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR26" t="inlineStr"/>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS26" t="inlineStr">
         <is>
           <t>Table 1</t>
@@ -4168,31 +3780,15 @@
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Meta-analysis</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Imaging</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>logistic regression (with covariates)</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
+          <t>meta-analysis + replication + discovery</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>SNP-based</t>
@@ -4200,30 +3796,22 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>ADSP</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>74046</t>
-        </is>
-      </c>
+          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>HRC;1000G</t>
+          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>European ancestry</t>
+          <t>european ancestry + adsp + adgc + eur</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
@@ -4232,7 +3820,11 @@
           <t>ADSP</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>ms4a6a + abca7 + alzheimers disease</t>
+        </is>
+      </c>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr"/>
@@ -4270,7 +3862,11 @@
           <t>30448613</t>
         </is>
       </c>
-      <c r="AR27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>PMC6331247</t>
+        </is>
+      </c>
       <c r="AS27" t="inlineStr">
         <is>
           <t>Table 1</t>

</xml_diff>

<commit_message>
Lower generated text to prevent extract weird info + add mapping to category of population, stage, and phenotyp
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU27"/>
+  <dimension ref="A1:AX27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -664,11 +664,26 @@
           <t>LocusName</t>
         </is>
       </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>Population category</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Stage category</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Phenotype category</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CR1</t>
+          <t>rs6656401</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -690,7 +705,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -703,7 +718,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -713,12 +728,12 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -729,7 +744,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -745,7 +760,11 @@
       <c r="AC2" t="n">
         <v>8.489999999999999e-07</v>
       </c>
-      <c r="AD2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
@@ -789,11 +808,26 @@
           <t>CR1</t>
         </is>
       </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CR1</t>
+          <t>rs4844600</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -815,7 +849,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -828,7 +862,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -838,12 +872,12 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -854,7 +888,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -870,7 +904,11 @@
       <c r="AC3" t="n">
         <v>4.219999999999999e-07</v>
       </c>
-      <c r="AD3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
@@ -914,9 +952,28 @@
           <t>CR1</t>
         </is>
       </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>rs2296160</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>30448613_table1_R00003</t>
@@ -936,7 +993,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -949,7 +1006,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -959,12 +1016,12 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -975,7 +1032,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -991,7 +1048,11 @@
       <c r="AC4" t="n">
         <v>4.24e-08</v>
       </c>
-      <c r="AD4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
@@ -1031,9 +1092,28 @@
         </is>
       </c>
       <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>rs2296160</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>30448613_table1_R00004</t>
@@ -1053,7 +1133,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1066,7 +1146,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1076,12 +1156,12 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1092,7 +1172,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -1108,7 +1188,11 @@
       <c r="AC5" t="n">
         <v>0.00856</v>
       </c>
-      <c r="AD5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
@@ -1148,11 +1232,26 @@
         </is>
       </c>
       <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HLA-DRB5</t>
+          <t>rs9271192</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1174,7 +1273,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1187,7 +1286,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1197,12 +1296,12 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1213,7 +1312,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -1229,7 +1328,11 @@
       <c r="AC6" t="n">
         <v>0.000266</v>
       </c>
-      <c r="AD6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
@@ -1273,11 +1376,26 @@
           <t>HLA-DRB5</t>
         </is>
       </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HLA-DRB5</t>
+          <t>rs9270303</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1299,7 +1417,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1312,7 +1430,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1322,12 +1440,12 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1338,7 +1456,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1354,7 +1472,11 @@
       <c r="AC7" t="n">
         <v>0.00025</v>
       </c>
-      <c r="AD7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
@@ -1398,11 +1520,26 @@
           <t>HLA-DRB5</t>
         </is>
       </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>rs1476679</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1424,7 +1561,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1437,7 +1574,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1447,12 +1584,12 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1463,7 +1600,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1479,7 +1616,11 @@
       <c r="AC8" t="n">
         <v>0.00141</v>
       </c>
-      <c r="AD8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
@@ -1523,11 +1664,26 @@
           <t>ZCWPW1</t>
         </is>
       </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>rs2405442</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1549,7 +1705,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1562,7 +1718,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1572,12 +1728,12 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1588,7 +1744,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1604,7 +1760,11 @@
       <c r="AC9" t="n">
         <v>0.00212</v>
       </c>
-      <c r="AD9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
@@ -1648,11 +1808,26 @@
           <t>ZCWPW1</t>
         </is>
       </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ZCWPW1</t>
+          <t>rs2405442</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1674,7 +1849,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1687,7 +1862,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1697,12 +1872,12 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1713,7 +1888,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1729,7 +1904,11 @@
       <c r="AC10" t="n">
         <v>0.00109</v>
       </c>
-      <c r="AD10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
@@ -1773,9 +1952,28 @@
           <t>ZCWPW1</t>
         </is>
       </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>rs1859788</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>30448613_table1_R00010</t>
@@ -1795,7 +1993,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1808,7 +2006,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1818,12 +2016,12 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -1834,7 +2032,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1850,7 +2048,11 @@
       <c r="AC11" t="n">
         <v>0.00562</v>
       </c>
-      <c r="AD11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
@@ -1890,9 +2092,28 @@
         </is>
       </c>
       <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>rs1859788</t>
+        </is>
+      </c>
       <c r="B12" t="inlineStr">
         <is>
           <t>30448613_table1_R00011</t>
@@ -1912,7 +2133,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1925,7 +2146,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1935,12 +2156,12 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -1951,7 +2172,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1967,7 +2188,11 @@
       <c r="AC12" t="n">
         <v>0.00112</v>
       </c>
-      <c r="AD12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
@@ -2007,11 +2232,26 @@
         </is>
       </c>
       <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>rs9331896</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2033,7 +2273,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2046,7 +2286,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -2056,12 +2296,12 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2072,7 +2312,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -2088,7 +2328,11 @@
       <c r="AC13" t="n">
         <v>0.00102</v>
       </c>
-      <c r="AD13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
@@ -2132,11 +2376,26 @@
           <t>CLU</t>
         </is>
       </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>rs7982</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2158,7 +2417,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2171,7 +2430,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2181,12 +2440,12 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2197,7 +2456,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -2213,7 +2472,11 @@
       <c r="AC14" t="n">
         <v>0.000364</v>
       </c>
-      <c r="AD14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
@@ -2257,11 +2520,26 @@
           <t>CLU</t>
         </is>
       </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CLU</t>
+          <t>rs7982</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2283,7 +2561,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2296,7 +2574,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2306,12 +2584,12 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2322,7 +2600,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -2338,7 +2616,11 @@
       <c r="AC15" t="n">
         <v>0.00162</v>
       </c>
-      <c r="AD15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
@@ -2382,11 +2664,26 @@
           <t>CLU</t>
         </is>
       </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>rs10838725</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2408,7 +2705,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2421,7 +2718,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2431,12 +2728,12 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2447,7 +2744,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -2463,7 +2760,11 @@
       <c r="AC16" t="n">
         <v>0.054</v>
       </c>
-      <c r="AD16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
@@ -2507,11 +2808,26 @@
           <t>CELF1</t>
         </is>
       </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>rs2293576</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2533,7 +2849,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2546,7 +2862,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2556,12 +2872,12 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2572,7 +2888,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -2588,7 +2904,11 @@
       <c r="AC17" t="n">
         <v>0.24</v>
       </c>
-      <c r="AD17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr"/>
       <c r="AG17" t="inlineStr"/>
@@ -2632,11 +2952,26 @@
           <t>CELF1</t>
         </is>
       </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CELF1</t>
+          <t>rs2293576</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2658,7 +2993,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -2671,7 +3006,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2681,12 +3016,12 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2697,7 +3032,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -2713,7 +3048,11 @@
       <c r="AC18" t="n">
         <v>0.04</v>
       </c>
-      <c r="AD18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
@@ -2757,11 +3096,26 @@
           <t>CELF1</t>
         </is>
       </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MS4A6A</t>
+          <t>rs983392</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2783,7 +3137,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -2796,7 +3150,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2806,12 +3160,12 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -2822,7 +3176,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -2838,7 +3192,11 @@
       <c r="AC19" t="n">
         <v>7.22e-09</v>
       </c>
-      <c r="AD19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
       <c r="AG19" t="inlineStr"/>
@@ -2882,11 +3240,26 @@
           <t>MS4A6A</t>
         </is>
       </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MS4A6A</t>
+          <t>rs12453</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2908,7 +3281,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -2921,7 +3294,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2931,12 +3304,12 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -2947,7 +3320,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -2963,7 +3336,11 @@
       <c r="AC20" t="n">
         <v>1.34e-09</v>
       </c>
-      <c r="AD20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="inlineStr"/>
@@ -3007,11 +3384,26 @@
           <t>MS4A6A</t>
         </is>
       </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MS4A6A</t>
+          <t>rs12453</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3033,7 +3425,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -3046,7 +3438,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -3056,12 +3448,12 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -3072,7 +3464,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -3088,7 +3480,11 @@
       <c r="AC21" t="n">
         <v>0.00036</v>
       </c>
-      <c r="AD21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr"/>
       <c r="AG21" t="inlineStr"/>
@@ -3132,11 +3528,26 @@
           <t>MS4A6A</t>
         </is>
       </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ABCA7</t>
+          <t>rs4147929</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3158,7 +3569,7 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -3171,7 +3582,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -3181,12 +3592,12 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3197,7 +3608,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -3213,7 +3624,11 @@
       <c r="AC22" t="n">
         <v>0.00139</v>
       </c>
-      <c r="AD22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr"/>
       <c r="AG22" t="inlineStr"/>
@@ -3257,11 +3672,26 @@
           <t>ABCA7</t>
         </is>
       </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW22" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ABCA7</t>
+          <t>rs3752246</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3283,7 +3713,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -3296,7 +3726,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -3306,12 +3736,12 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -3322,7 +3752,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -3338,7 +3768,11 @@
       <c r="AC23" t="n">
         <v>0.0027</v>
       </c>
-      <c r="AD23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
@@ -3382,11 +3816,26 @@
           <t>ABCA7</t>
         </is>
       </c>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW23" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ABCA7</t>
+          <t>rs3752246</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3408,7 +3857,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -3421,7 +3870,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -3431,12 +3880,12 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3447,7 +3896,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -3463,7 +3912,11 @@
       <c r="AC24" t="n">
         <v>9.890000000000002e-05</v>
       </c>
-      <c r="AD24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr"/>
       <c r="AG24" t="inlineStr"/>
@@ -3507,11 +3960,26 @@
           <t>ABCA7</t>
         </is>
       </c>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW24" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CD33</t>
+          <t>rs3865444</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3533,7 +4001,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -3546,7 +4014,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -3556,12 +4024,12 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3572,7 +4040,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -3588,7 +4056,11 @@
       <c r="AC25" t="n">
         <v>0.000449</v>
       </c>
-      <c r="AD25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>IGAP SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr"/>
       <c r="AG25" t="inlineStr"/>
@@ -3632,11 +4104,26 @@
           <t>CD33</t>
         </is>
       </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW25" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CD33</t>
+          <t>rs12459419</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3658,7 +4145,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -3671,7 +4158,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -3681,12 +4168,12 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -3697,7 +4184,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -3713,7 +4200,11 @@
       <c r="AC26" t="n">
         <v>0.000402</v>
       </c>
-      <c r="AD26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADGC P-value</t>
+        </is>
+      </c>
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr"/>
       <c r="AG26" t="inlineStr"/>
@@ -3757,11 +4248,26 @@
           <t>CD33</t>
         </is>
       </c>
+      <c r="AV26" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW26" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CD33</t>
+          <t>rs12459419</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3783,7 +4289,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>meta-analysis + replication + discovery</t>
+          <t>meta-analysis + discovery + replication + meta + combined</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -3796,7 +4302,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>CHARGE + ADSP + ADGC + UKBEC + IGAP + UKBB + ADNI + NABEC</t>
+          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -3806,12 +4312,12 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>hrc + hrc;1000g + topmed + igap + uk10k + 1000g</t>
+          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>european ancestry + adsp + adgc + eur</t>
+          <t>ethnic + adgc + race + european ancestry + ancestry</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
@@ -3822,7 +4328,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>ms4a6a + abca7 + alzheimers disease</t>
+          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -3838,7 +4344,11 @@
       <c r="AC27" t="n">
         <v>0.09</v>
       </c>
-      <c r="AD27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>Exonic SNP ADSP P-value</t>
+        </is>
+      </c>
       <c r="AE27" t="inlineStr"/>
       <c r="AF27" t="inlineStr"/>
       <c r="AG27" t="inlineStr"/>
@@ -3882,6 +4392,21 @@
           <t>CD33</t>
         </is>
       </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>Multi-ethnic</t>
+        </is>
+      </c>
+      <c r="AW27" t="inlineStr">
+        <is>
+          <t>Meta-analysis + Discovery + Replication</t>
+        </is>
+      </c>
+      <c r="AX27" t="inlineStr">
+        <is>
+          <t>AD (includes LOAD)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
use llama-server for faster inference
</commit_message>
<xml_diff>
--- a/harmonized_tables_advp/from_30448613_table1_v1.xlsx
+++ b/harmonized_tables_advp/from_30448613_table1_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX27"/>
+  <dimension ref="A1:AW27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -666,24 +666,19 @@
       </c>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>Population category</t>
+          <t>Population details</t>
         </is>
       </c>
       <c r="AW1" s="1" t="inlineStr">
         <is>
-          <t>Stage category</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>Phenotype category</t>
+          <t>Stage details</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>rs6656401</t>
+          <t>CR1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -705,7 +700,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -718,7 +713,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -728,12 +723,12 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -744,7 +739,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -760,11 +755,7 @@
       <c r="AC2" t="n">
         <v>8.489999999999999e-07</v>
       </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
@@ -810,24 +801,19 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rs4844600</t>
+          <t>CR1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -849,7 +835,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -862,7 +848,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -872,12 +858,12 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -888,7 +874,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -904,11 +890,7 @@
       <c r="AC3" t="n">
         <v>4.219999999999999e-07</v>
       </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
@@ -954,26 +936,17 @@
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>rs2296160</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>30448613_table1_R00003</t>
@@ -993,7 +966,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -1006,7 +979,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -1016,12 +989,12 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1032,7 +1005,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -1048,11 +1021,7 @@
       <c r="AC4" t="n">
         <v>4.24e-08</v>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
@@ -1094,26 +1063,17 @@
       <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>rs2296160</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>30448613_table1_R00004</t>
@@ -1133,7 +1093,7 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1146,7 +1106,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1156,12 +1116,12 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
@@ -1172,7 +1132,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
@@ -1188,11 +1148,7 @@
       <c r="AC5" t="n">
         <v>0.00856</v>
       </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
@@ -1234,24 +1190,19 @@
       <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rs9271192</t>
+          <t>HLA-DRB5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1273,7 +1224,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1286,7 +1237,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1296,12 +1247,12 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
@@ -1312,7 +1263,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -1328,11 +1279,7 @@
       <c r="AC6" t="n">
         <v>0.000266</v>
       </c>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
@@ -1378,24 +1325,19 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX6" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>rs9270303</t>
+          <t>HLA-DRB5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1417,7 +1359,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1430,7 +1372,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1440,12 +1382,12 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
@@ -1456,7 +1398,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1472,11 +1414,7 @@
       <c r="AC7" t="n">
         <v>0.00025</v>
       </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
@@ -1522,24 +1460,19 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX7" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>rs1476679</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1561,7 +1494,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1574,7 +1507,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1584,12 +1517,12 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
@@ -1600,7 +1533,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1616,11 +1549,7 @@
       <c r="AC8" t="n">
         <v>0.00141</v>
       </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
@@ -1666,24 +1595,19 @@
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX8" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rs2405442</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1705,7 +1629,7 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1718,7 +1642,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1728,12 +1652,12 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1744,7 +1668,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1760,11 +1684,7 @@
       <c r="AC9" t="n">
         <v>0.00212</v>
       </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
@@ -1810,24 +1730,19 @@
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX9" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rs2405442</t>
+          <t>ZCWPW1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1849,7 +1764,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1862,7 +1777,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1872,12 +1787,12 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -1888,7 +1803,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1904,11 +1819,7 @@
       <c r="AC10" t="n">
         <v>0.00109</v>
       </c>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
@@ -1954,26 +1865,17 @@
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX10" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>rs1859788</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>30448613_table1_R00010</t>
@@ -1993,7 +1895,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -2006,7 +1908,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -2016,12 +1918,12 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
@@ -2032,7 +1934,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -2048,11 +1950,7 @@
       <c r="AC11" t="n">
         <v>0.00562</v>
       </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
@@ -2094,26 +1992,17 @@
       <c r="AU11" t="inlineStr"/>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX11" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>rs1859788</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>30448613_table1_R00011</t>
@@ -2133,7 +2022,7 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -2146,7 +2035,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -2156,12 +2045,12 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -2172,7 +2061,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -2188,11 +2077,7 @@
       <c r="AC12" t="n">
         <v>0.00112</v>
       </c>
-      <c r="AD12" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
@@ -2234,24 +2119,19 @@
       <c r="AU12" t="inlineStr"/>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX12" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>rs9331896</t>
+          <t>CLU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2273,7 +2153,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -2286,7 +2166,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -2296,12 +2176,12 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -2312,7 +2192,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -2328,11 +2208,7 @@
       <c r="AC13" t="n">
         <v>0.00102</v>
       </c>
-      <c r="AD13" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
@@ -2378,24 +2254,19 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX13" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rs7982</t>
+          <t>CLU</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2417,7 +2288,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -2430,7 +2301,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2440,12 +2311,12 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
@@ -2456,7 +2327,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -2472,11 +2343,7 @@
       <c r="AC14" t="n">
         <v>0.000364</v>
       </c>
-      <c r="AD14" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
@@ -2522,24 +2389,19 @@
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX14" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>rs7982</t>
+          <t>CLU</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2561,7 +2423,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -2574,7 +2436,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -2584,12 +2446,12 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -2600,7 +2462,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -2616,11 +2478,7 @@
       <c r="AC15" t="n">
         <v>0.00162</v>
       </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
@@ -2666,24 +2524,19 @@
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX15" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>rs10838725</t>
+          <t>CELF1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2705,7 +2558,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -2718,7 +2571,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2728,12 +2581,12 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
@@ -2744,7 +2597,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -2760,11 +2613,7 @@
       <c r="AC16" t="n">
         <v>0.054</v>
       </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
@@ -2810,24 +2659,19 @@
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX16" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>rs2293576</t>
+          <t>CELF1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2849,7 +2693,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2862,7 +2706,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2872,12 +2716,12 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -2888,7 +2732,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -2904,11 +2748,7 @@
       <c r="AC17" t="n">
         <v>0.24</v>
       </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD17" t="inlineStr"/>
       <c r="AE17" t="inlineStr"/>
       <c r="AF17" t="inlineStr"/>
       <c r="AG17" t="inlineStr"/>
@@ -2954,24 +2794,19 @@
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX17" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>rs2293576</t>
+          <t>CELF1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2993,7 +2828,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -3006,7 +2841,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -3016,12 +2851,12 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -3032,7 +2867,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -3048,11 +2883,7 @@
       <c r="AC18" t="n">
         <v>0.04</v>
       </c>
-      <c r="AD18" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD18" t="inlineStr"/>
       <c r="AE18" t="inlineStr"/>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
@@ -3098,24 +2929,19 @@
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW18" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX18" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>rs983392</t>
+          <t>MS4A6A</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3137,7 +2963,7 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -3150,7 +2976,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -3160,12 +2986,12 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -3176,7 +3002,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -3192,11 +3018,7 @@
       <c r="AC19" t="n">
         <v>7.22e-09</v>
       </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="inlineStr"/>
       <c r="AF19" t="inlineStr"/>
       <c r="AG19" t="inlineStr"/>
@@ -3242,24 +3064,19 @@
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX19" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>rs12453</t>
+          <t>MS4A6A</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3281,7 +3098,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -3294,7 +3111,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -3304,12 +3121,12 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -3320,7 +3137,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -3336,11 +3153,7 @@
       <c r="AC20" t="n">
         <v>1.34e-09</v>
       </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD20" t="inlineStr"/>
       <c r="AE20" t="inlineStr"/>
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="inlineStr"/>
@@ -3386,24 +3199,19 @@
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX20" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>rs12453</t>
+          <t>MS4A6A</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3425,7 +3233,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -3438,7 +3246,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -3448,12 +3256,12 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -3464,7 +3272,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -3480,11 +3288,7 @@
       <c r="AC21" t="n">
         <v>0.00036</v>
       </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD21" t="inlineStr"/>
       <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="inlineStr"/>
       <c r="AG21" t="inlineStr"/>
@@ -3530,24 +3334,19 @@
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX21" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>rs4147929</t>
+          <t>ABCA7</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3569,7 +3368,7 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -3582,7 +3381,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -3592,12 +3391,12 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3608,7 +3407,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -3624,11 +3423,7 @@
       <c r="AC22" t="n">
         <v>0.00139</v>
       </c>
-      <c r="AD22" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD22" t="inlineStr"/>
       <c r="AE22" t="inlineStr"/>
       <c r="AF22" t="inlineStr"/>
       <c r="AG22" t="inlineStr"/>
@@ -3674,24 +3469,19 @@
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW22" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX22" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>rs3752246</t>
+          <t>ABCA7</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3713,7 +3503,7 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -3726,7 +3516,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -3736,12 +3526,12 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -3752,7 +3542,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -3768,11 +3558,7 @@
       <c r="AC23" t="n">
         <v>0.0027</v>
       </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD23" t="inlineStr"/>
       <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
@@ -3818,24 +3604,19 @@
       </c>
       <c r="AV23" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX23" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>rs3752246</t>
+          <t>ABCA7</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3857,7 +3638,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -3870,7 +3651,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -3880,12 +3661,12 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
@@ -3896,7 +3677,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -3912,11 +3693,7 @@
       <c r="AC24" t="n">
         <v>9.890000000000002e-05</v>
       </c>
-      <c r="AD24" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD24" t="inlineStr"/>
       <c r="AE24" t="inlineStr"/>
       <c r="AF24" t="inlineStr"/>
       <c r="AG24" t="inlineStr"/>
@@ -3962,24 +3739,19 @@
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW24" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX24" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>rs3865444</t>
+          <t>CD33</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4001,7 +3773,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -4014,7 +3786,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -4024,12 +3796,12 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -4040,7 +3812,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -4056,11 +3828,7 @@
       <c r="AC25" t="n">
         <v>0.000449</v>
       </c>
-      <c r="AD25" t="inlineStr">
-        <is>
-          <t>IGAP SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD25" t="inlineStr"/>
       <c r="AE25" t="inlineStr"/>
       <c r="AF25" t="inlineStr"/>
       <c r="AG25" t="inlineStr"/>
@@ -4106,24 +3874,19 @@
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX25" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>rs12459419</t>
+          <t>CD33</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4145,7 +3908,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -4158,7 +3921,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -4168,12 +3931,12 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -4184,7 +3947,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W26" t="inlineStr"/>
@@ -4200,11 +3963,7 @@
       <c r="AC26" t="n">
         <v>0.000402</v>
       </c>
-      <c r="AD26" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADGC P-value</t>
-        </is>
-      </c>
+      <c r="AD26" t="inlineStr"/>
       <c r="AE26" t="inlineStr"/>
       <c r="AF26" t="inlineStr"/>
       <c r="AG26" t="inlineStr"/>
@@ -4250,24 +4009,19 @@
       </c>
       <c r="AV26" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX26" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>rs12459419</t>
+          <t>CD33</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4289,7 +4043,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>meta-analysis + discovery + replication + meta + combined</t>
+          <t>Meta-analysis + Joint-analysis + Discovery + Replication</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -4302,7 +4056,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>adgc + discovery + 1000 genomes eur + adsp + study + international genomics of alzheimers project (igap)</t>
+          <t>adgc + adni.loni.usc.edu + adsp + international genomics of alzheimers project (igap) + charge + igap + adni</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -4312,12 +4066,12 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>rs9271192 + igap snps + 1000 genomes eur + adsp + hrc;1000g</t>
+          <t>1000 genome phase 3 v5 reference panel + adgc + eagle v2.3 phasing + maf + plink + d + igap snp + adsp + supplementary table 2 + charge + 1 mb + gcta + supplementary method + braineac + igap + michigan imputation server + hrc;1000g</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>ethnic + adgc + race + european ancestry + ancestry</t>
+          <t>asian + african american + multi-ethnic + caucasian + caribbean hispanic + european ancestry</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
@@ -4328,7 +4082,7 @@
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>alzheimers disease + ad + outcome + trait + ad phenotype + disease</t>
+          <t>synonymous mutations + cognitive decline + clusterin + tmem106b + amyloid beta peptide + presenilin 2 + alzheimers disease phenotype + alzheimer disease + rest and stress + alzheimers disease + dna repair + grn + alzheimers risk-altering polymorphism + kcnmb2 + abcc9 + hippocampal sclerosis of aging</t>
         </is>
       </c>
       <c r="W27" t="inlineStr"/>
@@ -4344,11 +4098,7 @@
       <c r="AC27" t="n">
         <v>0.09</v>
       </c>
-      <c r="AD27" t="inlineStr">
-        <is>
-          <t>Exonic SNP ADSP P-value</t>
-        </is>
-      </c>
+      <c r="AD27" t="inlineStr"/>
       <c r="AE27" t="inlineStr"/>
       <c r="AF27" t="inlineStr"/>
       <c r="AG27" t="inlineStr"/>
@@ -4394,17 +4144,12 @@
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>Multi-ethnic</t>
+          <t>race + adgc + pilra + european-type + ancestry + participant pools + ms4a6a + abca7 + clu + ethnic + hla-dqb1 + cr1 + nme8 + european ancestry</t>
         </is>
       </c>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>Meta-analysis + Discovery + Replication</t>
-        </is>
-      </c>
-      <c r="AX27" t="inlineStr">
-        <is>
-          <t>AD (includes LOAD)</t>
+          <t>discovery + replication + combined + meta-analyzing + meta</t>
         </is>
       </c>
     </row>

</xml_diff>